<commit_message>
feat: wire MIS test harness with real Aurora data, fix attendance page auth
- Populated test-harness/aurora-primary/ with real spreadsheets from Google Drive
  (420 pupils, 4620 attendance records, 5800 behaviour incidents, 360 statutory
  results, 1260 assessments, 84 SEN records, 89 teacher class assignments)
- Set MIS_DATA_SOURCE=local in env for dev (reads from test harness)
- Added MIS fallback to attendance dashboard API (reads real data when
  Supabase tables empty, before falling back to demo)
- Fixed attendance page: added organizationId to API URL
- Added test-harness/ to gitignore (contains real school data)
- Cleaned sidebar: workspace only has Home, My Tasks, Calendar

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/platform/test-harness/aurora-primary/arbor-exports/arbor_staff_export.xlsx
+++ b/apps/platform/test-harness/aurora-primary/arbor-exports/arbor_staff_export.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AO27"/>
+  <dimension ref="A1:U27"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,66 +463,6 @@
       <c r="U1" t="str">
         <v>Prevent Training</v>
       </c>
-      <c r="V1" t="str">
-        <v>Email</v>
-      </c>
-      <c r="W1" t="str">
-        <v>Phone</v>
-      </c>
-      <c r="X1" t="str">
-        <v>NI Number</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>TRN</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>Payroll Number</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>Hours Per Week</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>Weeks Per Year</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>Notice Period (Weeks)</v>
-      </c>
-      <c r="AD1" t="str">
-        <v>Continuous Service Date</v>
-      </c>
-      <c r="AE1" t="str">
-        <v>DBS Certificate Number</v>
-      </c>
-      <c r="AF1" t="str">
-        <v>DBS Update Service</v>
-      </c>
-      <c r="AG1" t="str">
-        <v>RTW Type</v>
-      </c>
-      <c r="AH1" t="str">
-        <v>RTW Check Date</v>
-      </c>
-      <c r="AI1" t="str">
-        <v>RTW Expiry</v>
-      </c>
-      <c r="AJ1" t="str">
-        <v>QTS Status</v>
-      </c>
-      <c r="AK1" t="str">
-        <v>First Aid Type</v>
-      </c>
-      <c r="AL1" t="str">
-        <v>First Aid Date</v>
-      </c>
-      <c r="AM1" t="str">
-        <v>First Aid Expiry</v>
-      </c>
-      <c r="AN1" t="str">
-        <v>Gender</v>
-      </c>
-      <c r="AO1" t="str">
-        <v>Date of Birth</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -588,66 +528,6 @@
       <c r="U2" t="str">
         <v>2024-10-01</v>
       </c>
-      <c r="V2" t="str">
-        <v>swilliams@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W2" t="str">
-        <v>07700100000</v>
-      </c>
-      <c r="X2" t="str">
-        <v>AB123456A</v>
-      </c>
-      <c r="Y2" t="str">
-        <v>1234567</v>
-      </c>
-      <c r="Z2" t="str">
-        <v>PAY1001</v>
-      </c>
-      <c r="AA2">
-        <v>32.5</v>
-      </c>
-      <c r="AB2">
-        <v>39</v>
-      </c>
-      <c r="AC2">
-        <v>8</v>
-      </c>
-      <c r="AD2" t="str">
-        <v>2013-09-01</v>
-      </c>
-      <c r="AE2" t="str">
-        <v>100000000000</v>
-      </c>
-      <c r="AF2" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG2" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH2" t="str">
-        <v>2015-09-01</v>
-      </c>
-      <c r="AI2" t="str">
-        <v/>
-      </c>
-      <c r="AJ2" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK2" t="str">
-        <v/>
-      </c>
-      <c r="AL2" t="str">
-        <v/>
-      </c>
-      <c r="AM2" t="str">
-        <v/>
-      </c>
-      <c r="AN2" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO2" t="str">
-        <v>1965-01-05</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -713,66 +593,6 @@
       <c r="U3" t="str">
         <v>2024-04-01</v>
       </c>
-      <c r="V3" t="str">
-        <v>jthompson@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W3" t="str">
-        <v>07711107919</v>
-      </c>
-      <c r="X3" t="str">
-        <v>CD134567A</v>
-      </c>
-      <c r="Y3" t="str">
-        <v>1245678</v>
-      </c>
-      <c r="Z3" t="str">
-        <v>PAY1002</v>
-      </c>
-      <c r="AA3">
-        <v>32.5</v>
-      </c>
-      <c r="AB3">
-        <v>39</v>
-      </c>
-      <c r="AC3">
-        <v>8</v>
-      </c>
-      <c r="AD3" t="str">
-        <v>2017-09-01</v>
-      </c>
-      <c r="AE3" t="str">
-        <v>108761234567</v>
-      </c>
-      <c r="AF3" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG3" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH3" t="str">
-        <v>2017-09-01</v>
-      </c>
-      <c r="AI3" t="str">
-        <v/>
-      </c>
-      <c r="AJ3" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK3" t="str">
-        <v/>
-      </c>
-      <c r="AL3" t="str">
-        <v/>
-      </c>
-      <c r="AM3" t="str">
-        <v/>
-      </c>
-      <c r="AN3" t="str">
-        <v>Male</v>
-      </c>
-      <c r="AO3" t="str">
-        <v>1968-02-06</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -838,66 +658,6 @@
       <c r="U4" t="str">
         <v>2024-12-01</v>
       </c>
-      <c r="V4" t="str">
-        <v>mrobinson@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W4" t="str">
-        <v>07722115838</v>
-      </c>
-      <c r="X4" t="str">
-        <v>EF145678A</v>
-      </c>
-      <c r="Y4" t="str">
-        <v>1256789</v>
-      </c>
-      <c r="Z4" t="str">
-        <v>PAY1003</v>
-      </c>
-      <c r="AA4">
-        <v>27.5</v>
-      </c>
-      <c r="AB4">
-        <v>39</v>
-      </c>
-      <c r="AC4">
-        <v>8</v>
-      </c>
-      <c r="AD4" t="str">
-        <v>2014-09-01</v>
-      </c>
-      <c r="AE4" t="str">
-        <v>117522469134</v>
-      </c>
-      <c r="AF4" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG4" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH4" t="str">
-        <v>2016-09-01</v>
-      </c>
-      <c r="AI4" t="str">
-        <v/>
-      </c>
-      <c r="AJ4" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK4" t="str">
-        <v>Paediatric First Aid</v>
-      </c>
-      <c r="AL4" t="str">
-        <v>2025-06-15</v>
-      </c>
-      <c r="AM4" t="str">
-        <v>2028-06-15</v>
-      </c>
-      <c r="AN4" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO4" t="str">
-        <v>1971-03-07</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -963,66 +723,6 @@
       <c r="U5" t="str">
         <v>2025-01-01</v>
       </c>
-      <c r="V5" t="str">
-        <v>dclark@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W5" t="str">
-        <v>07733123757</v>
-      </c>
-      <c r="X5" t="str">
-        <v>GH156789A</v>
-      </c>
-      <c r="Y5" t="str">
-        <v>1267900</v>
-      </c>
-      <c r="Z5" t="str">
-        <v>PAY1004</v>
-      </c>
-      <c r="AA5">
-        <v>32.5</v>
-      </c>
-      <c r="AB5">
-        <v>39</v>
-      </c>
-      <c r="AC5">
-        <v>8</v>
-      </c>
-      <c r="AD5" t="str">
-        <v>2023-09-01</v>
-      </c>
-      <c r="AE5" t="str">
-        <v>126283703701</v>
-      </c>
-      <c r="AF5" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG5" t="str">
-        <v>EU Settled Status</v>
-      </c>
-      <c r="AH5" t="str">
-        <v>2024-09-01</v>
-      </c>
-      <c r="AI5" t="str">
-        <v>2028-06-30</v>
-      </c>
-      <c r="AJ5" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK5" t="str">
-        <v/>
-      </c>
-      <c r="AL5" t="str">
-        <v/>
-      </c>
-      <c r="AM5" t="str">
-        <v/>
-      </c>
-      <c r="AN5" t="str">
-        <v>Male</v>
-      </c>
-      <c r="AO5" t="str">
-        <v>1974-04-08</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1088,66 +788,6 @@
       <c r="U6" t="str">
         <v>2024-05-01</v>
       </c>
-      <c r="V6" t="str">
-        <v>aturner@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W6" t="str">
-        <v>07744131676</v>
-      </c>
-      <c r="X6" t="str">
-        <v>JK167900A</v>
-      </c>
-      <c r="Y6" t="str">
-        <v>1279011</v>
-      </c>
-      <c r="Z6" t="str">
-        <v>PAY1005</v>
-      </c>
-      <c r="AA6">
-        <v>32.5</v>
-      </c>
-      <c r="AB6">
-        <v>39</v>
-      </c>
-      <c r="AC6">
-        <v>8</v>
-      </c>
-      <c r="AD6" t="str">
-        <v>2019-09-01</v>
-      </c>
-      <c r="AE6" t="str">
-        <v>135044938268</v>
-      </c>
-      <c r="AF6" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG6" t="str">
-        <v>British Birth Certificate</v>
-      </c>
-      <c r="AH6" t="str">
-        <v>2020-09-01</v>
-      </c>
-      <c r="AI6" t="str">
-        <v/>
-      </c>
-      <c r="AJ6" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK6" t="str">
-        <v>Emergency First Aid</v>
-      </c>
-      <c r="AL6" t="str">
-        <v>2025-06-15</v>
-      </c>
-      <c r="AM6" t="str">
-        <v>2028-06-15</v>
-      </c>
-      <c r="AN6" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO6" t="str">
-        <v>1977-05-09</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1213,66 +853,6 @@
       <c r="U7" t="str">
         <v>2024-05-01</v>
       </c>
-      <c r="V7" t="str">
-        <v>nharris@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W7" t="str">
-        <v>07755139595</v>
-      </c>
-      <c r="X7" t="str">
-        <v>LM179011A</v>
-      </c>
-      <c r="Y7" t="str">
-        <v>1290122</v>
-      </c>
-      <c r="Z7" t="str">
-        <v>PAY1006</v>
-      </c>
-      <c r="AA7">
-        <v>32.5</v>
-      </c>
-      <c r="AB7">
-        <v>39</v>
-      </c>
-      <c r="AC7">
-        <v>8</v>
-      </c>
-      <c r="AD7" t="str">
-        <v>2021-09-01</v>
-      </c>
-      <c r="AE7" t="str">
-        <v>143806172835</v>
-      </c>
-      <c r="AF7" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG7" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH7" t="str">
-        <v>2021-09-01</v>
-      </c>
-      <c r="AI7" t="str">
-        <v/>
-      </c>
-      <c r="AJ7" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK7" t="str">
-        <v/>
-      </c>
-      <c r="AL7" t="str">
-        <v/>
-      </c>
-      <c r="AM7" t="str">
-        <v/>
-      </c>
-      <c r="AN7" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO7" t="str">
-        <v>1980-06-10</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1338,66 +918,6 @@
       <c r="U8" t="str">
         <v>2025-10-01</v>
       </c>
-      <c r="V8" t="str">
-        <v>lwalker@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W8" t="str">
-        <v>07766147514</v>
-      </c>
-      <c r="X8" t="str">
-        <v>NP190122A</v>
-      </c>
-      <c r="Y8" t="str">
-        <v>1301233</v>
-      </c>
-      <c r="Z8" t="str">
-        <v>PAY1007</v>
-      </c>
-      <c r="AA8">
-        <v>32.5</v>
-      </c>
-      <c r="AB8">
-        <v>39</v>
-      </c>
-      <c r="AC8">
-        <v>8</v>
-      </c>
-      <c r="AD8" t="str">
-        <v>2018-09-01</v>
-      </c>
-      <c r="AE8" t="str">
-        <v>152567407402</v>
-      </c>
-      <c r="AF8" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG8" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH8" t="str">
-        <v>2018-09-01</v>
-      </c>
-      <c r="AI8" t="str">
-        <v/>
-      </c>
-      <c r="AJ8" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK8" t="str">
-        <v/>
-      </c>
-      <c r="AL8" t="str">
-        <v/>
-      </c>
-      <c r="AM8" t="str">
-        <v/>
-      </c>
-      <c r="AN8" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO8" t="str">
-        <v>1983-07-11</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -1463,66 +983,6 @@
       <c r="U9" t="str">
         <v>2025-12-01</v>
       </c>
-      <c r="V9" t="str">
-        <v>kmorgan@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W9" t="str">
-        <v>07777155433</v>
-      </c>
-      <c r="X9" t="str">
-        <v>RS201233A</v>
-      </c>
-      <c r="Y9" t="str">
-        <v>1312344</v>
-      </c>
-      <c r="Z9" t="str">
-        <v>PAY1008</v>
-      </c>
-      <c r="AA9">
-        <v>19.5</v>
-      </c>
-      <c r="AB9">
-        <v>39</v>
-      </c>
-      <c r="AC9">
-        <v>8</v>
-      </c>
-      <c r="AD9" t="str">
-        <v>2014-09-01</v>
-      </c>
-      <c r="AE9" t="str">
-        <v>161328641969</v>
-      </c>
-      <c r="AF9" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG9" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH9" t="str">
-        <v>2014-09-01</v>
-      </c>
-      <c r="AI9" t="str">
-        <v/>
-      </c>
-      <c r="AJ9" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK9" t="str">
-        <v/>
-      </c>
-      <c r="AL9" t="str">
-        <v/>
-      </c>
-      <c r="AM9" t="str">
-        <v/>
-      </c>
-      <c r="AN9" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO9" t="str">
-        <v>1986-08-12</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -1588,66 +1048,6 @@
       <c r="U10" t="str">
         <v>2024-06-01</v>
       </c>
-      <c r="V10" t="str">
-        <v>pdavis@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W10" t="str">
-        <v>07788163352</v>
-      </c>
-      <c r="X10" t="str">
-        <v>TW212344A</v>
-      </c>
-      <c r="Y10" t="str">
-        <v>1323455</v>
-      </c>
-      <c r="Z10" t="str">
-        <v>PAY1009</v>
-      </c>
-      <c r="AA10">
-        <v>32.5</v>
-      </c>
-      <c r="AB10">
-        <v>39</v>
-      </c>
-      <c r="AC10">
-        <v>8</v>
-      </c>
-      <c r="AD10" t="str">
-        <v>2017-09-01</v>
-      </c>
-      <c r="AE10" t="str">
-        <v>170089876536</v>
-      </c>
-      <c r="AF10" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG10" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH10" t="str">
-        <v>2019-09-01</v>
-      </c>
-      <c r="AI10" t="str">
-        <v/>
-      </c>
-      <c r="AJ10" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK10" t="str">
-        <v>Paediatric First Aid</v>
-      </c>
-      <c r="AL10" t="str">
-        <v>2025-06-15</v>
-      </c>
-      <c r="AM10" t="str">
-        <v>2028-06-15</v>
-      </c>
-      <c r="AN10" t="str">
-        <v>Male</v>
-      </c>
-      <c r="AO10" t="str">
-        <v>1989-09-13</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -1713,66 +1113,6 @@
       <c r="U11" t="str">
         <v>2025-11-01</v>
       </c>
-      <c r="V11" t="str">
-        <v>awilson@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W11" t="str">
-        <v>07799171271</v>
-      </c>
-      <c r="X11" t="str">
-        <v>YZ223455A</v>
-      </c>
-      <c r="Y11" t="str">
-        <v>1334566</v>
-      </c>
-      <c r="Z11" t="str">
-        <v>PAY1010</v>
-      </c>
-      <c r="AA11">
-        <v>32.5</v>
-      </c>
-      <c r="AB11">
-        <v>39</v>
-      </c>
-      <c r="AC11">
-        <v>8</v>
-      </c>
-      <c r="AD11" t="str">
-        <v>2016-09-01</v>
-      </c>
-      <c r="AE11" t="str">
-        <v>178851111103</v>
-      </c>
-      <c r="AF11" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG11" t="str">
-        <v>EU Settled Status</v>
-      </c>
-      <c r="AH11" t="str">
-        <v>2016-09-01</v>
-      </c>
-      <c r="AI11" t="str">
-        <v>2028-06-30</v>
-      </c>
-      <c r="AJ11" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK11" t="str">
-        <v/>
-      </c>
-      <c r="AL11" t="str">
-        <v/>
-      </c>
-      <c r="AM11" t="str">
-        <v/>
-      </c>
-      <c r="AN11" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO11" t="str">
-        <v>1992-10-14</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1838,66 +1178,6 @@
       <c r="U12" t="str">
         <v>2024-08-01</v>
       </c>
-      <c r="V12" t="str">
-        <v>sbrown@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W12" t="str">
-        <v>07810179190</v>
-      </c>
-      <c r="X12" t="str">
-        <v>AB234566A</v>
-      </c>
-      <c r="Y12" t="str">
-        <v>1345677</v>
-      </c>
-      <c r="Z12" t="str">
-        <v>PAY1011</v>
-      </c>
-      <c r="AA12">
-        <v>32.5</v>
-      </c>
-      <c r="AB12">
-        <v>39</v>
-      </c>
-      <c r="AC12">
-        <v>8</v>
-      </c>
-      <c r="AD12" t="str">
-        <v>2018-09-01</v>
-      </c>
-      <c r="AE12" t="str">
-        <v>187612345670</v>
-      </c>
-      <c r="AF12" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG12" t="str">
-        <v>British Birth Certificate</v>
-      </c>
-      <c r="AH12" t="str">
-        <v>2019-09-01</v>
-      </c>
-      <c r="AI12" t="str">
-        <v/>
-      </c>
-      <c r="AJ12" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK12" t="str">
-        <v/>
-      </c>
-      <c r="AL12" t="str">
-        <v/>
-      </c>
-      <c r="AM12" t="str">
-        <v/>
-      </c>
-      <c r="AN12" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO12" t="str">
-        <v>1965-11-15</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1963,66 +1243,6 @@
       <c r="U13" t="str">
         <v>2025-05-01</v>
       </c>
-      <c r="V13" t="str">
-        <v>ctaylor@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W13" t="str">
-        <v>07821187109</v>
-      </c>
-      <c r="X13" t="str">
-        <v>CD245677A</v>
-      </c>
-      <c r="Y13" t="str">
-        <v>1356788</v>
-      </c>
-      <c r="Z13" t="str">
-        <v>PAY1012</v>
-      </c>
-      <c r="AA13">
-        <v>32.5</v>
-      </c>
-      <c r="AB13">
-        <v>39</v>
-      </c>
-      <c r="AC13">
-        <v>8</v>
-      </c>
-      <c r="AD13" t="str">
-        <v>2013-09-01</v>
-      </c>
-      <c r="AE13" t="str">
-        <v>196373580237</v>
-      </c>
-      <c r="AF13" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG13" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH13" t="str">
-        <v>2013-09-01</v>
-      </c>
-      <c r="AI13" t="str">
-        <v/>
-      </c>
-      <c r="AJ13" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK13" t="str">
-        <v/>
-      </c>
-      <c r="AL13" t="str">
-        <v/>
-      </c>
-      <c r="AM13" t="str">
-        <v/>
-      </c>
-      <c r="AN13" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO13" t="str">
-        <v>1968-12-16</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -2088,66 +1308,6 @@
       <c r="U14" t="str">
         <v>2024-07-01</v>
       </c>
-      <c r="V14" t="str">
-        <v>rmartinez@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W14" t="str">
-        <v>07832195028</v>
-      </c>
-      <c r="X14" t="str">
-        <v>EF256788A</v>
-      </c>
-      <c r="Y14" t="str">
-        <v>1367899</v>
-      </c>
-      <c r="Z14" t="str">
-        <v>PAY1013</v>
-      </c>
-      <c r="AA14">
-        <v>32.5</v>
-      </c>
-      <c r="AB14">
-        <v>39</v>
-      </c>
-      <c r="AC14">
-        <v>8</v>
-      </c>
-      <c r="AD14" t="str">
-        <v>2018-09-01</v>
-      </c>
-      <c r="AE14" t="str">
-        <v>205134814804</v>
-      </c>
-      <c r="AF14" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG14" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH14" t="str">
-        <v>2018-09-01</v>
-      </c>
-      <c r="AI14" t="str">
-        <v/>
-      </c>
-      <c r="AJ14" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK14" t="str">
-        <v>Paediatric First Aid</v>
-      </c>
-      <c r="AL14" t="str">
-        <v>2025-06-15</v>
-      </c>
-      <c r="AM14" t="str">
-        <v>2028-06-15</v>
-      </c>
-      <c r="AN14" t="str">
-        <v>Male</v>
-      </c>
-      <c r="AO14" t="str">
-        <v>1971-01-17</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -2213,66 +1373,6 @@
       <c r="U15" t="str">
         <v>2025-04-01</v>
       </c>
-      <c r="V15" t="str">
-        <v>janderson@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W15" t="str">
-        <v>07843202947</v>
-      </c>
-      <c r="X15" t="str">
-        <v>GH267899A</v>
-      </c>
-      <c r="Y15" t="str">
-        <v>1379010</v>
-      </c>
-      <c r="Z15" t="str">
-        <v>PAY1014</v>
-      </c>
-      <c r="AA15">
-        <v>32.5</v>
-      </c>
-      <c r="AB15">
-        <v>39</v>
-      </c>
-      <c r="AC15">
-        <v>8</v>
-      </c>
-      <c r="AD15" t="str">
-        <v>2018-09-01</v>
-      </c>
-      <c r="AE15" t="str">
-        <v>213896049371</v>
-      </c>
-      <c r="AF15" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG15" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH15" t="str">
-        <v>2019-09-01</v>
-      </c>
-      <c r="AI15" t="str">
-        <v/>
-      </c>
-      <c r="AJ15" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK15" t="str">
-        <v/>
-      </c>
-      <c r="AL15" t="str">
-        <v/>
-      </c>
-      <c r="AM15" t="str">
-        <v/>
-      </c>
-      <c r="AN15" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO15" t="str">
-        <v>1974-02-18</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -2338,66 +1438,6 @@
       <c r="U16" t="str">
         <v>2025-03-01</v>
       </c>
-      <c r="V16" t="str">
-        <v>hthomas@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W16" t="str">
-        <v>07854210866</v>
-      </c>
-      <c r="X16" t="str">
-        <v>JK279010A</v>
-      </c>
-      <c r="Y16" t="str">
-        <v>1390121</v>
-      </c>
-      <c r="Z16" t="str">
-        <v>PAY1015</v>
-      </c>
-      <c r="AA16">
-        <v>32.5</v>
-      </c>
-      <c r="AB16">
-        <v>39</v>
-      </c>
-      <c r="AC16">
-        <v>8</v>
-      </c>
-      <c r="AD16" t="str">
-        <v>2016-09-01</v>
-      </c>
-      <c r="AE16" t="str">
-        <v>222657283938</v>
-      </c>
-      <c r="AF16" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG16" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH16" t="str">
-        <v>2017-09-01</v>
-      </c>
-      <c r="AI16" t="str">
-        <v/>
-      </c>
-      <c r="AJ16" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK16" t="str">
-        <v>Emergency First Aid</v>
-      </c>
-      <c r="AL16" t="str">
-        <v>2025-06-15</v>
-      </c>
-      <c r="AM16" t="str">
-        <v>2028-06-15</v>
-      </c>
-      <c r="AN16" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO16" t="str">
-        <v>1977-03-19</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -2463,66 +1503,6 @@
       <c r="U17" t="str">
         <v>2024-12-01</v>
       </c>
-      <c r="V17" t="str">
-        <v>fjackson@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W17" t="str">
-        <v>07865218785</v>
-      </c>
-      <c r="X17" t="str">
-        <v>LM290121A</v>
-      </c>
-      <c r="Y17" t="str">
-        <v>1401232</v>
-      </c>
-      <c r="Z17" t="str">
-        <v>PAY1016</v>
-      </c>
-      <c r="AA17">
-        <v>19.5</v>
-      </c>
-      <c r="AB17">
-        <v>39</v>
-      </c>
-      <c r="AC17">
-        <v>8</v>
-      </c>
-      <c r="AD17" t="str">
-        <v>2019-09-01</v>
-      </c>
-      <c r="AE17" t="str">
-        <v>231418518505</v>
-      </c>
-      <c r="AF17" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG17" t="str">
-        <v>EU Settled Status</v>
-      </c>
-      <c r="AH17" t="str">
-        <v>2020-09-01</v>
-      </c>
-      <c r="AI17" t="str">
-        <v>2028-06-30</v>
-      </c>
-      <c r="AJ17" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK17" t="str">
-        <v/>
-      </c>
-      <c r="AL17" t="str">
-        <v/>
-      </c>
-      <c r="AM17" t="str">
-        <v/>
-      </c>
-      <c r="AN17" t="str">
-        <v>Male</v>
-      </c>
-      <c r="AO17" t="str">
-        <v>1980-04-20</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -2588,66 +1568,6 @@
       <c r="U18" t="str">
         <v>2025-10-01</v>
       </c>
-      <c r="V18" t="str">
-        <v>bwhite@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W18" t="str">
-        <v>07876226704</v>
-      </c>
-      <c r="X18" t="str">
-        <v>NP301232A</v>
-      </c>
-      <c r="Y18" t="str">
-        <v>1412343</v>
-      </c>
-      <c r="Z18" t="str">
-        <v>PAY1017</v>
-      </c>
-      <c r="AA18">
-        <v>32.5</v>
-      </c>
-      <c r="AB18">
-        <v>39</v>
-      </c>
-      <c r="AC18">
-        <v>8</v>
-      </c>
-      <c r="AD18" t="str">
-        <v>2011-09-01</v>
-      </c>
-      <c r="AE18" t="str">
-        <v>240179753072</v>
-      </c>
-      <c r="AF18" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG18" t="str">
-        <v>British Birth Certificate</v>
-      </c>
-      <c r="AH18" t="str">
-        <v>2011-09-01</v>
-      </c>
-      <c r="AI18" t="str">
-        <v/>
-      </c>
-      <c r="AJ18" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK18" t="str">
-        <v/>
-      </c>
-      <c r="AL18" t="str">
-        <v/>
-      </c>
-      <c r="AM18" t="str">
-        <v/>
-      </c>
-      <c r="AN18" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO18" t="str">
-        <v>1983-05-21</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -2713,66 +1633,6 @@
       <c r="U19" t="str">
         <v>2024-02-01</v>
       </c>
-      <c r="V19" t="str">
-        <v>gmartin@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W19" t="str">
-        <v>07887234623</v>
-      </c>
-      <c r="X19" t="str">
-        <v>RS312343A</v>
-      </c>
-      <c r="Y19" t="str">
-        <v/>
-      </c>
-      <c r="Z19" t="str">
-        <v>PAY1018</v>
-      </c>
-      <c r="AA19">
-        <v>32.5</v>
-      </c>
-      <c r="AB19">
-        <v>52</v>
-      </c>
-      <c r="AC19">
-        <v>4</v>
-      </c>
-      <c r="AD19" t="str">
-        <v>2017-01-08</v>
-      </c>
-      <c r="AE19" t="str">
-        <v>248940987639</v>
-      </c>
-      <c r="AF19" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG19" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH19" t="str">
-        <v>2018-01-08</v>
-      </c>
-      <c r="AI19" t="str">
-        <v/>
-      </c>
-      <c r="AJ19" t="str">
-        <v/>
-      </c>
-      <c r="AK19" t="str">
-        <v/>
-      </c>
-      <c r="AL19" t="str">
-        <v/>
-      </c>
-      <c r="AM19" t="str">
-        <v/>
-      </c>
-      <c r="AN19" t="str">
-        <v>Male</v>
-      </c>
-      <c r="AO19" t="str">
-        <v>1986-06-22</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -2838,66 +1698,6 @@
       <c r="U20" t="str">
         <v>2024-05-01</v>
       </c>
-      <c r="V20" t="str">
-        <v>elee@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W20" t="str">
-        <v>07898242542</v>
-      </c>
-      <c r="X20" t="str">
-        <v>TW323454A</v>
-      </c>
-      <c r="Y20" t="str">
-        <v/>
-      </c>
-      <c r="Z20" t="str">
-        <v>PAY1019</v>
-      </c>
-      <c r="AA20">
-        <v>37</v>
-      </c>
-      <c r="AB20">
-        <v>52</v>
-      </c>
-      <c r="AC20">
-        <v>4</v>
-      </c>
-      <c r="AD20" t="str">
-        <v>2011-04-01</v>
-      </c>
-      <c r="AE20" t="str">
-        <v>257702222206</v>
-      </c>
-      <c r="AF20" t="str">
-        <v>No</v>
-      </c>
-      <c r="AG20" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH20" t="str">
-        <v>2012-04-01</v>
-      </c>
-      <c r="AI20" t="str">
-        <v/>
-      </c>
-      <c r="AJ20" t="str">
-        <v/>
-      </c>
-      <c r="AK20" t="str">
-        <v>Paediatric First Aid</v>
-      </c>
-      <c r="AL20" t="str">
-        <v>2025-06-15</v>
-      </c>
-      <c r="AM20" t="str">
-        <v>2028-06-15</v>
-      </c>
-      <c r="AN20" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO20" t="str">
-        <v>1989-07-23</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -2963,66 +1763,6 @@
       <c r="U21" t="str">
         <v>2025-01-01</v>
       </c>
-      <c r="V21" t="str">
-        <v>dwilliams@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W21" t="str">
-        <v>07909250461</v>
-      </c>
-      <c r="X21" t="str">
-        <v>YZ334565A</v>
-      </c>
-      <c r="Y21" t="str">
-        <v/>
-      </c>
-      <c r="Z21" t="str">
-        <v>PAY1020</v>
-      </c>
-      <c r="AA21">
-        <v>27.5</v>
-      </c>
-      <c r="AB21">
-        <v>39</v>
-      </c>
-      <c r="AC21">
-        <v>4</v>
-      </c>
-      <c r="AD21" t="str">
-        <v>2014-09-01</v>
-      </c>
-      <c r="AE21" t="str">
-        <v>266463456773</v>
-      </c>
-      <c r="AF21" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG21" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH21" t="str">
-        <v>2015-09-01</v>
-      </c>
-      <c r="AI21" t="str">
-        <v/>
-      </c>
-      <c r="AJ21" t="str">
-        <v/>
-      </c>
-      <c r="AK21" t="str">
-        <v/>
-      </c>
-      <c r="AL21" t="str">
-        <v/>
-      </c>
-      <c r="AM21" t="str">
-        <v/>
-      </c>
-      <c r="AN21" t="str">
-        <v>Male</v>
-      </c>
-      <c r="AO21" t="str">
-        <v>1992-08-24</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -3088,66 +1828,6 @@
       <c r="U22" t="str">
         <v>2025-04-01</v>
       </c>
-      <c r="V22" t="str">
-        <v>spatel@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W22" t="str">
-        <v>07920258380</v>
-      </c>
-      <c r="X22" t="str">
-        <v>AB345676A</v>
-      </c>
-      <c r="Y22" t="str">
-        <v/>
-      </c>
-      <c r="Z22" t="str">
-        <v>PAY1021</v>
-      </c>
-      <c r="AA22">
-        <v>27.5</v>
-      </c>
-      <c r="AB22">
-        <v>39</v>
-      </c>
-      <c r="AC22">
-        <v>4</v>
-      </c>
-      <c r="AD22" t="str">
-        <v>2021-09-01</v>
-      </c>
-      <c r="AE22" t="str">
-        <v>275224691340</v>
-      </c>
-      <c r="AF22" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG22" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH22" t="str">
-        <v>2022-09-01</v>
-      </c>
-      <c r="AI22" t="str">
-        <v/>
-      </c>
-      <c r="AJ22" t="str">
-        <v/>
-      </c>
-      <c r="AK22" t="str">
-        <v/>
-      </c>
-      <c r="AL22" t="str">
-        <v/>
-      </c>
-      <c r="AM22" t="str">
-        <v/>
-      </c>
-      <c r="AN22" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO22" t="str">
-        <v>1965-09-05</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -3213,66 +1893,6 @@
       <c r="U23" t="str">
         <v>2024-04-01</v>
       </c>
-      <c r="V23" t="str">
-        <v>jallen@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W23" t="str">
-        <v>07931266299</v>
-      </c>
-      <c r="X23" t="str">
-        <v>CD356787A</v>
-      </c>
-      <c r="Y23" t="str">
-        <v>1467898</v>
-      </c>
-      <c r="Z23" t="str">
-        <v>PAY1022</v>
-      </c>
-      <c r="AA23">
-        <v>13</v>
-      </c>
-      <c r="AB23">
-        <v>39</v>
-      </c>
-      <c r="AC23">
-        <v>8</v>
-      </c>
-      <c r="AD23" t="str">
-        <v>2012-09-01</v>
-      </c>
-      <c r="AE23" t="str">
-        <v>283985925907</v>
-      </c>
-      <c r="AF23" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG23" t="str">
-        <v>EU Settled Status</v>
-      </c>
-      <c r="AH23" t="str">
-        <v>2014-09-01</v>
-      </c>
-      <c r="AI23" t="str">
-        <v>2028-06-30</v>
-      </c>
-      <c r="AJ23" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK23" t="str">
-        <v/>
-      </c>
-      <c r="AL23" t="str">
-        <v/>
-      </c>
-      <c r="AM23" t="str">
-        <v/>
-      </c>
-      <c r="AN23" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO23" t="str">
-        <v>1968-10-06</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -3338,66 +1958,6 @@
       <c r="U24" t="str">
         <v>2024-12-01</v>
       </c>
-      <c r="V24" t="str">
-        <v>myoung@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W24" t="str">
-        <v>07942274218</v>
-      </c>
-      <c r="X24" t="str">
-        <v>EF367898A</v>
-      </c>
-      <c r="Y24" t="str">
-        <v>1479009</v>
-      </c>
-      <c r="Z24" t="str">
-        <v>PAY1023</v>
-      </c>
-      <c r="AA24">
-        <v>0</v>
-      </c>
-      <c r="AB24">
-        <v>39</v>
-      </c>
-      <c r="AC24">
-        <v>8</v>
-      </c>
-      <c r="AD24" t="str">
-        <v>2024-09-02</v>
-      </c>
-      <c r="AE24" t="str">
-        <v>292747160474</v>
-      </c>
-      <c r="AF24" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG24" t="str">
-        <v>British Birth Certificate</v>
-      </c>
-      <c r="AH24" t="str">
-        <v>2024-09-02</v>
-      </c>
-      <c r="AI24" t="str">
-        <v/>
-      </c>
-      <c r="AJ24" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK24" t="str">
-        <v>Paediatric First Aid</v>
-      </c>
-      <c r="AL24" t="str">
-        <v>2025-06-15</v>
-      </c>
-      <c r="AM24" t="str">
-        <v>2028-06-15</v>
-      </c>
-      <c r="AN24" t="str">
-        <v>Male</v>
-      </c>
-      <c r="AO24" t="str">
-        <v>1971-11-07</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -3463,66 +2023,6 @@
       <c r="U25" t="str">
         <v>2025-09-01</v>
       </c>
-      <c r="V25" t="str">
-        <v>tking@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W25" t="str">
-        <v>07953282137</v>
-      </c>
-      <c r="X25" t="str">
-        <v>GH379009A</v>
-      </c>
-      <c r="Y25" t="str">
-        <v>1490120</v>
-      </c>
-      <c r="Z25" t="str">
-        <v>PAY1024</v>
-      </c>
-      <c r="AA25">
-        <v>0</v>
-      </c>
-      <c r="AB25">
-        <v>39</v>
-      </c>
-      <c r="AC25">
-        <v>8</v>
-      </c>
-      <c r="AD25" t="str">
-        <v>2024-01-06</v>
-      </c>
-      <c r="AE25" t="str">
-        <v>301508395041</v>
-      </c>
-      <c r="AF25" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="AG25" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH25" t="str">
-        <v>2025-01-06</v>
-      </c>
-      <c r="AI25" t="str">
-        <v/>
-      </c>
-      <c r="AJ25" t="str">
-        <v>Qualified</v>
-      </c>
-      <c r="AK25" t="str">
-        <v/>
-      </c>
-      <c r="AL25" t="str">
-        <v/>
-      </c>
-      <c r="AM25" t="str">
-        <v/>
-      </c>
-      <c r="AN25" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO25" t="str">
-        <v>1974-12-08</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -3588,66 +2088,6 @@
       <c r="U26" t="str">
         <v>2025-03-01</v>
       </c>
-      <c r="V26" t="str">
-        <v>awright@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W26" t="str">
-        <v>07964290056</v>
-      </c>
-      <c r="X26" t="str">
-        <v>JK390120A</v>
-      </c>
-      <c r="Y26" t="str">
-        <v/>
-      </c>
-      <c r="Z26" t="str">
-        <v>PAY1025</v>
-      </c>
-      <c r="AA26">
-        <v>27.5</v>
-      </c>
-      <c r="AB26">
-        <v>39</v>
-      </c>
-      <c r="AC26">
-        <v>4</v>
-      </c>
-      <c r="AD26" t="str">
-        <v>2017-09-01</v>
-      </c>
-      <c r="AE26" t="str">
-        <v>310269629608</v>
-      </c>
-      <c r="AF26" t="str">
-        <v>No</v>
-      </c>
-      <c r="AG26" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH26" t="str">
-        <v>2019-09-01</v>
-      </c>
-      <c r="AI26" t="str">
-        <v/>
-      </c>
-      <c r="AJ26" t="str">
-        <v/>
-      </c>
-      <c r="AK26" t="str">
-        <v>Emergency First Aid</v>
-      </c>
-      <c r="AL26" t="str">
-        <v>2025-06-15</v>
-      </c>
-      <c r="AM26" t="str">
-        <v>2028-06-15</v>
-      </c>
-      <c r="AN26" t="str">
-        <v>Male</v>
-      </c>
-      <c r="AO26" t="str">
-        <v>1977-01-09</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -3713,70 +2153,10 @@
       <c r="U27" t="str">
         <v>2025-01-01</v>
       </c>
-      <c r="V27" t="str">
-        <v>cscott@aurora-primary.schoolgle.co.uk</v>
-      </c>
-      <c r="W27" t="str">
-        <v>07975297975</v>
-      </c>
-      <c r="X27" t="str">
-        <v>LM401231A</v>
-      </c>
-      <c r="Y27" t="str">
-        <v/>
-      </c>
-      <c r="Z27" t="str">
-        <v>PAY1026</v>
-      </c>
-      <c r="AA27">
-        <v>27.5</v>
-      </c>
-      <c r="AB27">
-        <v>39</v>
-      </c>
-      <c r="AC27">
-        <v>4</v>
-      </c>
-      <c r="AD27" t="str">
-        <v>2019-09-01</v>
-      </c>
-      <c r="AE27" t="str">
-        <v>319030864175</v>
-      </c>
-      <c r="AF27" t="str">
-        <v>No</v>
-      </c>
-      <c r="AG27" t="str">
-        <v>British Passport</v>
-      </c>
-      <c r="AH27" t="str">
-        <v>2021-09-01</v>
-      </c>
-      <c r="AI27" t="str">
-        <v/>
-      </c>
-      <c r="AJ27" t="str">
-        <v/>
-      </c>
-      <c r="AK27" t="str">
-        <v/>
-      </c>
-      <c r="AL27" t="str">
-        <v/>
-      </c>
-      <c r="AM27" t="str">
-        <v/>
-      </c>
-      <c r="AN27" t="str">
-        <v>Female</v>
-      </c>
-      <c r="AO27" t="str">
-        <v>1980-02-10</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AO27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ed): integrate Ed chatbot with bottom-left positioning, personalised greetings, data isolation
- Move Ed widget to bottom-left with sidebar offset (CSS override)
- Enable real ed-widget package (remove stub alias in next.config.ts)
- Fix widget API auth: add credentials: "include" to fetch calls
- Personalised greetings: first name, time-of-day, domain-aware openers
- Conversation continuity: ed_conversation_log table (topics only, no PII)
- Role-based data access rules injected into every specialist prompt
- Organisation lookup via organization_members (proper multi-tenant)
- Ed enable/disable per school via organization_settings
- Screen capture + image upload support in EdSidebarChat fallback component
- EdChatbotProvider children now optional for dashboard-only rendering

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/platform/test-harness/aurora-primary/arbor-exports/arbor_staff_export.xlsx
+++ b/apps/platform/test-harness/aurora-primary/arbor-exports/arbor_staff_export.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2154,9 +2154,659 @@
         <v>2025-01-01</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>STF-027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Lisa</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Ahmed</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Teaching Assistant (1:1 EHCP)</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v>SC4</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Y2 Ash</v>
+      </c>
+      <c r="J28" t="str">
+        <v>2021-09-01</v>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="M28">
+        <v>2</v>
+      </c>
+      <c r="N28">
+        <v>1</v>
+      </c>
+      <c r="O28">
+        <v>2</v>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+      <c r="R28" t="str">
+        <v>Enhanced</v>
+      </c>
+      <c r="S28" t="str">
+        <v>2021-08-15</v>
+      </c>
+      <c r="T28" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U28" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>STF-028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Ms</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Ngozi</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Okafor</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Teaching Assistant (1:1 EHCP)</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v>SC4</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Y3 Holly</v>
+      </c>
+      <c r="J29" t="str">
+        <v>2023-09-01</v>
+      </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
+      <c r="L29" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="M29">
+        <v>4</v>
+      </c>
+      <c r="N29">
+        <v>2</v>
+      </c>
+      <c r="O29">
+        <v>16</v>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
+      <c r="R29" t="str">
+        <v>Enhanced</v>
+      </c>
+      <c r="S29" t="str">
+        <v>2023-08-20</v>
+      </c>
+      <c r="T29" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U29" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>STF-029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Samira</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Khan</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Teaching Assistant (1:1 EHCP)</v>
+      </c>
+      <c r="F30">
+        <v>1</v>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v>SC4</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Y4 Cedar</v>
+      </c>
+      <c r="J30" t="str">
+        <v>2022-09-01</v>
+      </c>
+      <c r="K30" t="str">
+        <v/>
+      </c>
+      <c r="L30" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="M30">
+        <v>1</v>
+      </c>
+      <c r="N30">
+        <v>1</v>
+      </c>
+      <c r="O30">
+        <v>1</v>
+      </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
+      <c r="R30" t="str">
+        <v>Enhanced</v>
+      </c>
+      <c r="S30" t="str">
+        <v>2022-08-10</v>
+      </c>
+      <c r="T30" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U30" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>STF-030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Jade</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Williams</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Teaching Assistant</v>
+      </c>
+      <c r="F31">
+        <v>1</v>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v>SC3</v>
+      </c>
+      <c r="I31" t="str">
+        <v>R Oak/Maple</v>
+      </c>
+      <c r="J31" t="str">
+        <v>2020-09-01</v>
+      </c>
+      <c r="K31" t="str">
+        <v/>
+      </c>
+      <c r="L31" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="M31">
+        <v>3</v>
+      </c>
+      <c r="N31">
+        <v>1</v>
+      </c>
+      <c r="O31">
+        <v>3</v>
+      </c>
+      <c r="P31" t="str">
+        <v/>
+      </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
+      <c r="R31" t="str">
+        <v>Enhanced</v>
+      </c>
+      <c r="S31" t="str">
+        <v>2020-08-12</v>
+      </c>
+      <c r="T31" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U31" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>STF-031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Daniel</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Cooper</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Teaching Assistant (1:1 EHCP)</v>
+      </c>
+      <c r="F32">
+        <v>1</v>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+      <c r="H32" t="str">
+        <v>SC4</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Y6 Sycamore</v>
+      </c>
+      <c r="J32" t="str">
+        <v>2023-09-01</v>
+      </c>
+      <c r="K32" t="str">
+        <v/>
+      </c>
+      <c r="L32" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="M32">
+        <v>6</v>
+      </c>
+      <c r="N32">
+        <v>2</v>
+      </c>
+      <c r="O32">
+        <v>24</v>
+      </c>
+      <c r="P32" t="str">
+        <v/>
+      </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
+      <c r="R32" t="str">
+        <v>Enhanced</v>
+      </c>
+      <c r="S32" t="str">
+        <v>2023-08-18</v>
+      </c>
+      <c r="T32" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U32" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>STF-032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Hannah</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Morris</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Teaching Assistant</v>
+      </c>
+      <c r="F33">
+        <v>0.8</v>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v>SC3</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Y3/Y4</v>
+      </c>
+      <c r="J33" t="str">
+        <v>2018-09-01</v>
+      </c>
+      <c r="K33" t="str">
+        <v/>
+      </c>
+      <c r="L33" t="str">
+        <v>Part-Time</v>
+      </c>
+      <c r="M33">
+        <v>2</v>
+      </c>
+      <c r="N33">
+        <v>1</v>
+      </c>
+      <c r="O33">
+        <v>2</v>
+      </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
+      <c r="R33" t="str">
+        <v>Enhanced</v>
+      </c>
+      <c r="S33" t="str">
+        <v>2018-08-22</v>
+      </c>
+      <c r="T33" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U33" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>STF-033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Julie</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Carter</v>
+      </c>
+      <c r="E34" t="str">
+        <v>HLTA</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <v>SC5</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Y1/Y2 PPA Cover</v>
+      </c>
+      <c r="J34" t="str">
+        <v>2015-09-01</v>
+      </c>
+      <c r="K34" t="str">
+        <v/>
+      </c>
+      <c r="L34" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="M34">
+        <v>1</v>
+      </c>
+      <c r="N34">
+        <v>1</v>
+      </c>
+      <c r="O34">
+        <v>1</v>
+      </c>
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
+      <c r="R34" t="str">
+        <v>Enhanced</v>
+      </c>
+      <c r="S34" t="str">
+        <v>2015-08-20</v>
+      </c>
+      <c r="T34" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U34" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>STF-034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Becky</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Turner</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Teaching Assistant (1:1 EHCP)</v>
+      </c>
+      <c r="F35">
+        <v>1</v>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <v>SC4</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Y2 Willow</v>
+      </c>
+      <c r="J35" t="str">
+        <v>2024-09-01</v>
+      </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
+      <c r="L35" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="M35">
+        <v>0</v>
+      </c>
+      <c r="N35">
+        <v>0</v>
+      </c>
+      <c r="O35">
+        <v>0</v>
+      </c>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
+      <c r="R35" t="str">
+        <v>Enhanced</v>
+      </c>
+      <c r="S35" t="str">
+        <v>2024-08-15</v>
+      </c>
+      <c r="T35" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U35" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>STF-035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Anita</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Sharma</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Teaching Assistant (1:1 EHCP)</v>
+      </c>
+      <c r="F36">
+        <v>1</v>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v>SC4</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Y1 Birch</v>
+      </c>
+      <c r="J36" t="str">
+        <v>2022-01-10</v>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
+      <c r="L36" t="str">
+        <v>Permanent</v>
+      </c>
+      <c r="M36">
+        <v>3</v>
+      </c>
+      <c r="N36">
+        <v>2</v>
+      </c>
+      <c r="O36">
+        <v>12</v>
+      </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
+      <c r="R36" t="str">
+        <v>Enhanced</v>
+      </c>
+      <c r="S36" t="str">
+        <v>2022-01-05</v>
+      </c>
+      <c r="T36" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U36" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>STF-036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Paula</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Dixon</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Teaching Assistant</v>
+      </c>
+      <c r="F37">
+        <v>0.6</v>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v>SC3</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Y6 Hazel/Sycamore</v>
+      </c>
+      <c r="J37" t="str">
+        <v>2019-09-01</v>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v>Part-Time</v>
+      </c>
+      <c r="M37">
+        <v>5</v>
+      </c>
+      <c r="N37">
+        <v>2</v>
+      </c>
+      <c r="O37">
+        <v>20</v>
+      </c>
+      <c r="P37" t="str">
+        <v/>
+      </c>
+      <c r="Q37" t="str">
+        <v/>
+      </c>
+      <c r="R37" t="str">
+        <v>Enhanced</v>
+      </c>
+      <c r="S37" t="str">
+        <v>2019-08-20</v>
+      </c>
+      <c r="T37" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U37" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>